<commit_message>
Update manual step reasons: remove B2B reason for step 10, note that steps 17-18 work on mcstaging Staging 1
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Staging2_Remediation_Updated.xlsx
+++ b/docs/GlobeWest_Staging2_Remediation_Updated.xlsx
@@ -746,7 +746,7 @@
         <v>MANUAL</v>
       </c>
       <c r="H13" t="str">
-        <v>MANUAL – B2B session required. CAPTCHA blocks automation.</v>
+        <v>MANUAL – CAPTCHA blocks automation. Verify fields and keyboard echo.</v>
       </c>
     </row>
     <row r="14" ht="40" customHeight="1">
@@ -928,7 +928,7 @@
         <v>MANUAL</v>
       </c>
       <c r="H20" t="str">
-        <v>MANUAL – Reseller must be pre-assigned in Staging 2 DB</v>
+        <v>MANUAL – Blocked on mcstaging2 (works perfectly on mcstaging Staging 1, payment successful)</v>
       </c>
     </row>
     <row r="21" ht="40" customHeight="1">
@@ -954,7 +954,7 @@
         <v>MANUAL</v>
       </c>
       <c r="H21" t="str">
-        <v>MANUAL – Depends on Step 17 completion</v>
+        <v>MANUAL – Blocked on mcstaging2 (works perfectly on mcstaging Staging 1)</v>
       </c>
     </row>
   </sheetData>
@@ -1096,7 +1096,7 @@
         <v>Enter "name your order" and "client name"</v>
       </c>
       <c r="C3" t="str" xml:space="preserve">
-        <v xml:space="preserve">B2B customer checkout fields — Requires logged-in B2B account. CAPTCHA blocks automation.
+        <v xml:space="preserve">CAPTCHA blocks automation.
 Manual: Check label announced by NVDA, echo typed characters.</v>
       </c>
       <c r="D3" t="str">
@@ -1111,8 +1111,8 @@
         <v>Confirm the order (Place Order)</v>
       </c>
       <c r="C4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Reseller must be pre-assigned in Staging 2 database.
-Place Order button is not enabled until valid reseller is assigned.
+        <v xml:space="preserve">Blocked on mcstaging2 (Place Order button is not enabled due to no reseller assigned for postcode 3000 in Staging 2 DB).
+Note: This step works perfectly on mcstaging (Staging 1).
 Manual: Verify T&amp;Cs keyboard + NVDA announcement + button activation.</v>
       </c>
       <c r="D4" t="str">
@@ -1127,7 +1127,8 @@
         <v>Review order confirmation</v>
       </c>
       <c r="C5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Depends on Step 17 manual completion.
+        <v xml:space="preserve">Blocked on mcstaging2 (depends on Step 17 placement).
+Note: This step works perfectly on mcstaging (Staging 1) order confirmation page.
 Manual: Verify NVDA reads order confirmation heading and order number clearly.</v>
       </c>
       <c r="D5" t="str">

</xml_diff>